<commit_message>
case 3 ver code and results -gaussblur3x3 int shift
</commit_message>
<xml_diff>
--- a/filter-cases/final_img/metrics_3x3.xlsx
+++ b/filter-cases/final_img/metrics_3x3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6138CB-D000-47B0-9999-660792931CA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9917E48B-1540-4928-9835-F5410350143F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29316" yWindow="2508" windowWidth="26796" windowHeight="12264" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
+    <workbookView xWindow="-28452" yWindow="3756" windowWidth="26796" windowHeight="12264" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
   <si>
     <t>sobel3x3_int_shift</t>
   </si>
@@ -153,6 +153,12 @@
   </si>
   <si>
     <t>366x485</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_rec_gaussblur3x3_int_shift</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_out_gaussblur3x3_int_shift</t>
   </si>
 </sst>
 </file>
@@ -564,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7225027-CB40-48EE-B4E7-9AA397931008}">
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -844,6 +850,72 @@
         <v>1</v>
       </c>
     </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>0.46595796942710799</v>
+      </c>
+      <c r="F11">
+        <v>0.68261116743087702</v>
+      </c>
+      <c r="G11">
+        <v>0.99896690452025805</v>
+      </c>
+      <c r="H11">
+        <v>51.447336220525997</v>
+      </c>
+      <c r="I11">
+        <v>2320</v>
+      </c>
+      <c r="J11">
+        <v>6093</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>4.6230000000000002</v>
+      </c>
+      <c r="N11">
+        <v>737</v>
+      </c>
+      <c r="O11">
+        <v>177512</v>
+      </c>
+      <c r="P11">
+        <f>N11+($F$2*$E$2)</f>
+        <v>176549</v>
+      </c>
+      <c r="Q11">
+        <f>1000/(T11-M11)</f>
+        <v>119.37447773665991</v>
+      </c>
+      <c r="R11">
+        <f t="shared" ref="R10:R11" si="0">U11*Q11</f>
+        <v>119.37447773665991</v>
+      </c>
+      <c r="S11">
+        <f>Q11*10^6/P11</f>
+        <v>676.15493566465921</v>
+      </c>
+      <c r="T11">
+        <v>13</v>
+      </c>
+      <c r="U11">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
gaussian blur 3x3 ieee - ver code and results
</commit_message>
<xml_diff>
--- a/filter-cases/final_img/metrics_3x3.xlsx
+++ b/filter-cases/final_img/metrics_3x3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9917E48B-1540-4928-9835-F5410350143F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790DA77A-231C-4B8F-87AB-5C2EBED0F5B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28452" yWindow="3756" windowWidth="26796" windowHeight="12264" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>sobel3x3_int_shift</t>
   </si>
@@ -159,6 +159,18 @@
   </si>
   <si>
     <t>smeagol_verilog_out_gaussblur3x3_int_shift</t>
+  </si>
+  <si>
+    <t>gaussblur3x3_ieee</t>
+  </si>
+  <si>
+    <t>gaussblur3x3_int_shift</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_rec_gaussblur3x3_ieee</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_out_gaussblur3x3_ieee</t>
   </si>
 </sst>
 </file>
@@ -570,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7225027-CB40-48EE-B4E7-9AA397931008}">
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -851,6 +863,9 @@
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
       <c r="B11" t="s">
         <v>39</v>
       </c>
@@ -902,7 +917,7 @@
         <v>119.37447773665991</v>
       </c>
       <c r="R11">
-        <f t="shared" ref="R10:R11" si="0">U11*Q11</f>
+        <f t="shared" ref="R10:R12" si="0">U11*Q11</f>
         <v>119.37447773665991</v>
       </c>
       <c r="S11">
@@ -913,6 +928,75 @@
         <v>13</v>
       </c>
       <c r="U11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>0.46595796942710799</v>
+      </c>
+      <c r="F12">
+        <v>0.68261116743087702</v>
+      </c>
+      <c r="G12">
+        <v>0.99896690452025805</v>
+      </c>
+      <c r="H12">
+        <v>51.447336220525997</v>
+      </c>
+      <c r="I12">
+        <v>7739</v>
+      </c>
+      <c r="J12">
+        <v>6565</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>12</v>
+      </c>
+      <c r="M12">
+        <v>1.101</v>
+      </c>
+      <c r="N12">
+        <v>742</v>
+      </c>
+      <c r="O12">
+        <v>177517</v>
+      </c>
+      <c r="P12">
+        <f>N12+($F$2*$E$2)</f>
+        <v>176554</v>
+      </c>
+      <c r="Q12">
+        <f>1000/(T12-M12)</f>
+        <v>84.040675687032518</v>
+      </c>
+      <c r="R12">
+        <f>U12*Q12</f>
+        <v>84.040675687032518</v>
+      </c>
+      <c r="S12">
+        <f>Q12*10^6/P12</f>
+        <v>476.00550362513746</v>
+      </c>
+      <c r="T12">
+        <v>13</v>
+      </c>
+      <c r="U12">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cascade3x3 int code and results
</commit_message>
<xml_diff>
--- a/filter-cases/final_img/metrics_3x3.xlsx
+++ b/filter-cases/final_img/metrics_3x3.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790DA77A-231C-4B8F-87AB-5C2EBED0F5B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2377BBD1-D1F9-48A0-A380-9B4FE993A7D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28452" yWindow="3756" windowWidth="26796" windowHeight="12264" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
+    <workbookView xWindow="1320" yWindow="1320" windowWidth="18098" windowHeight="7103" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
   <si>
     <t>sobel3x3_int_shift</t>
   </si>
@@ -171,6 +172,15 @@
   </si>
   <si>
     <t>smeagol_verilog_out_gaussblur3x3_ieee</t>
+  </si>
+  <si>
+    <t>cascade_3x3_int_shift</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_out_cascade_3x3_int_shift</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_rec_cascade_3x3_int_shift</t>
   </si>
 </sst>
 </file>
@@ -582,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7225027-CB40-48EE-B4E7-9AA397931008}">
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -917,7 +927,7 @@
         <v>119.37447773665991</v>
       </c>
       <c r="R11">
-        <f t="shared" ref="R10:R12" si="0">U11*Q11</f>
+        <f t="shared" ref="R11" si="0">U11*Q11</f>
         <v>119.37447773665991</v>
       </c>
       <c r="S11">
@@ -997,6 +1007,75 @@
         <v>13</v>
       </c>
       <c r="U12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14">
+        <v>6</v>
+      </c>
+      <c r="E14">
+        <v>5.2477874755859304</v>
+      </c>
+      <c r="F14">
+        <v>2.2908051013946502</v>
+      </c>
+      <c r="G14">
+        <v>0.99291031001720997</v>
+      </c>
+      <c r="H14">
+        <v>40.931041264318701</v>
+      </c>
+      <c r="I14">
+        <v>4722</v>
+      </c>
+      <c r="J14">
+        <v>12233</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>3.5950000000000002</v>
+      </c>
+      <c r="N14">
+        <v>1481</v>
+      </c>
+      <c r="O14">
+        <v>179220</v>
+      </c>
+      <c r="P14">
+        <f t="shared" ref="P13:P14" si="1">N14+($F$2*$E$2)</f>
+        <v>177293</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" ref="Q13:Q14" si="2">1000/(T14-M14)</f>
+        <v>106.32642211589581</v>
+      </c>
+      <c r="R14">
+        <f t="shared" ref="R13:R14" si="3">U14*Q14</f>
+        <v>106.32642211589581</v>
+      </c>
+      <c r="S14">
+        <f t="shared" ref="S13:S14" si="4">Q14*10^6/P14</f>
+        <v>599.72148993979351</v>
+      </c>
+      <c r="T14">
+        <v>13</v>
+      </c>
+      <c r="U14">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cascade3x3 ieee code and results
</commit_message>
<xml_diff>
--- a/filter-cases/final_img/metrics_3x3.xlsx
+++ b/filter-cases/final_img/metrics_3x3.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\fysiko_apth\ptuxiaki\thesis-cases\final_img\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2377BBD1-D1F9-48A0-A380-9B4FE993A7D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F17019D-D9DC-4312-A07C-AE2D975BF53C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="1320" windowWidth="18098" windowHeight="7103" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
+    <workbookView xWindow="-30132" yWindow="588" windowWidth="23040" windowHeight="11976" xr2:uid="{1A5AD2DC-DE0B-4FFA-AE19-FC07F326EFA1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
   <si>
     <t>sobel3x3_int_shift</t>
   </si>
@@ -181,6 +180,15 @@
   </si>
   <si>
     <t>smeagol_verilog_rec_cascade_3x3_int_shift</t>
+  </si>
+  <si>
+    <t>cascade_3x3_ieee</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_out_cascade_3x3_ieee</t>
+  </si>
+  <si>
+    <t>smeagol_verilog_rec_cascade_3x3_ieee</t>
   </si>
 </sst>
 </file>
@@ -592,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7225027-CB40-48EE-B4E7-9AA397931008}">
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
@@ -1057,25 +1065,94 @@
         <v>179220</v>
       </c>
       <c r="P14">
-        <f t="shared" ref="P13:P14" si="1">N14+($F$2*$E$2)</f>
+        <f t="shared" ref="P14:P15" si="1">N14+($F$2*$E$2)</f>
         <v>177293</v>
       </c>
       <c r="Q14">
-        <f t="shared" ref="Q13:Q14" si="2">1000/(T14-M14)</f>
+        <f t="shared" ref="Q14:Q15" si="2">1000/(T14-M14)</f>
         <v>106.32642211589581</v>
       </c>
       <c r="R14">
-        <f t="shared" ref="R13:R14" si="3">U14*Q14</f>
+        <f t="shared" ref="R14:R15" si="3">U14*Q14</f>
         <v>106.32642211589581</v>
       </c>
       <c r="S14">
-        <f t="shared" ref="S13:S14" si="4">Q14*10^6/P14</f>
+        <f t="shared" ref="S14:S15" si="4">Q14*10^6/P14</f>
         <v>599.72148993979351</v>
       </c>
       <c r="T14">
         <v>13</v>
       </c>
       <c r="U14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15">
+        <v>6</v>
+      </c>
+      <c r="E15">
+        <v>5.2477874755859304</v>
+      </c>
+      <c r="F15">
+        <v>2.2908051013946502</v>
+      </c>
+      <c r="G15">
+        <v>0.99291031001720997</v>
+      </c>
+      <c r="H15">
+        <v>40.931041264318701</v>
+      </c>
+      <c r="I15">
+        <v>17962</v>
+      </c>
+      <c r="J15">
+        <v>13384</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>32</v>
+      </c>
+      <c r="M15">
+        <v>0.77200000000000002</v>
+      </c>
+      <c r="N15">
+        <v>1490</v>
+      </c>
+      <c r="O15">
+        <v>179229</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="1"/>
+        <v>177302</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="2"/>
+        <v>81.779522407589141</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="3"/>
+        <v>81.779522407589141</v>
+      </c>
+      <c r="S15">
+        <f t="shared" si="4"/>
+        <v>461.24421838213408</v>
+      </c>
+      <c r="T15">
+        <v>13</v>
+      </c>
+      <c r="U15">
         <v>1</v>
       </c>
     </row>

</xml_diff>